<commit_message>
docs: update project academic team members across documentation and spreadsheets
</commit_message>
<xml_diff>
--- a/projeto-semestral/Documento de metrificação - Vitalis.xlsx
+++ b/projeto-semestral/Documento de metrificação - Vitalis.xlsx
@@ -1222,10 +1222,10 @@
     <ns0:t>HOSPITAL UNIVERSITÁRIO VITALIS / UCSAL</ns0:t>
   </ns0:si>
   <ns0:si>
-    <ns0:t>SISTEMA DE GESTÃO HOSPITALAR INTELIGENTE VITALIS (VERSÃO 2.0)</ns0:t>
-  </ns0:si>
-  <ns0:si>
-    <ns0:t>DAVI DOS SANTOS RIBEIRO</ns0:t>
+    <ns0:t>SISTEMA DE GESTÃO HOSPITALAR INTELIGENTE VITALIS</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Alisson de Oliveira dos Santos, Davi dos Santos Ribeiro, Larissa da Silva Santana, Maria Fernanda Pereira Barçante Costa, Rafael Farias Castro</ns0:t>
   </ns0:si>
   <ns0:si>
     <ns0:t>MFI-01: Cadastro de Pacientes, Validação CNS/CPF e Recepção</ns0:t>

</xml_diff>